<commit_message>
Update reports 2026-10-29 10:06
</commit_message>
<xml_diff>
--- a/gex_pivot_levels_2026-10-29.xlsx
+++ b/gex_pivot_levels_2026-10-29.xlsx
@@ -606,12 +606,12 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>-$6.07M</t>
+          <t>-$6.76M</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>+$6.54M</t>
+          <t>+$7.25M</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
@@ -639,12 +639,12 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>-$1.71M</t>
+          <t>-$1.76M</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>+$2.37M</t>
+          <t>+$2.45M</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -672,12 +672,12 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>-$8.65M</t>
+          <t>-$9.17M</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>+$11.50M</t>
+          <t>+$12.20M</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
@@ -738,12 +738,12 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>-$1.62M</t>
+          <t>-$1.66M</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>+$8.88M</t>
+          <t>+$9.07M</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
@@ -804,12 +804,12 @@
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>-$16.70M</t>
+          <t>-$16.48M</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>+$40.44M</t>
+          <t>+$39.90M</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
@@ -870,12 +870,12 @@
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>+$561.75K</t>
+          <t>+$547.34K</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>+$7.62M</t>
+          <t>+$7.42M</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
@@ -903,12 +903,12 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>-$4.14M</t>
+          <t>-$4.04M</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>+$10.24M</t>
+          <t>+$9.99M</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -969,12 +969,12 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>-$3.95M</t>
+          <t>-$3.85M</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>+$21.70M</t>
+          <t>+$21.18M</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
@@ -998,12 +998,12 @@
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>+$7.82M</t>
+          <t>+$7.59M</t>
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>+$23.22M</t>
+          <t>+$22.53M</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
@@ -1031,12 +1031,12 @@
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>+$1.73M</t>
+          <t>+$1.70M</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>+$5.62M</t>
+          <t>+$5.52M</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
@@ -1097,12 +1097,12 @@
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>+$8.02M</t>
+          <t>+$7.83M</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>+$11.11M</t>
+          <t>+$10.84M</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
@@ -1130,12 +1130,12 @@
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
-          <t>+$1.05M</t>
+          <t>+$1.02M</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>+$4.25M</t>
+          <t>+$4.09M</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
@@ -1275,7 +1275,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>28686.7</v>
+        <v>28732.95</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>705</v>
@@ -1304,7 +1304,7 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>28809.96</v>
+        <v>28856.21</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>708</v>
@@ -1333,7 +1333,7 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>28892.13</v>
+        <v>28938.38</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>710</v>
@@ -1362,7 +1362,7 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>29056.48</v>
+        <v>29102.73</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>714</v>
@@ -1395,7 +1395,7 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>29097.57</v>
+        <v>29143.82</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>715</v>
@@ -1424,7 +1424,7 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>29138.65</v>
+        <v>29184.9</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>716</v>
@@ -1457,7 +1457,7 @@
     </row>
     <row r="8">
       <c r="A8" s="5" t="n">
-        <v>29220.83</v>
+        <v>29267.08</v>
       </c>
       <c r="B8" s="5" t="n">
         <v>718</v>
@@ -1490,7 +1490,7 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>29261.92</v>
+        <v>29308.17</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>719</v>
@@ -1523,7 +1523,7 @@
     </row>
     <row r="10">
       <c r="A10" s="5" t="n">
-        <v>29303</v>
+        <v>29349.25</v>
       </c>
       <c r="B10" s="5" t="n">
         <v>720</v>
@@ -1556,7 +1556,7 @@
     </row>
     <row r="11">
       <c r="A11" s="5" t="n">
-        <v>29380.34</v>
+        <v>29426.59</v>
       </c>
       <c r="B11" s="5" t="n">
         <v>29660</v>
@@ -1589,7 +1589,7 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>29385.18</v>
+        <v>29431.43</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>722</v>
@@ -1618,7 +1618,7 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>29410.34</v>
+        <v>29456.59</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>29690</v>
@@ -1651,7 +1651,7 @@
     </row>
     <row r="14">
       <c r="A14" s="5" t="n">
-        <v>29440.34</v>
+        <v>29486.59</v>
       </c>
       <c r="B14" s="5" t="n">
         <v>29720</v>
@@ -1684,7 +1684,7 @@
     </row>
     <row r="15">
       <c r="A15" s="5" t="n">
-        <v>29508.44</v>
+        <v>29554.69</v>
       </c>
       <c r="B15" s="5" t="n">
         <v>725</v>
@@ -1717,7 +1717,7 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>29510.34</v>
+        <v>29556.59</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>29790</v>
@@ -1750,7 +1750,7 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>29530.34</v>
+        <v>29576.59</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>29810</v>
@@ -1779,7 +1779,7 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>29590.61</v>
+        <v>29636.86</v>
       </c>
       <c r="B18" s="2" t="n">
         <v>727</v>
@@ -1808,7 +1808,7 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="n">
-        <v>29630.34</v>
+        <v>29676.59</v>
       </c>
       <c r="B19" s="5" t="n">
         <v>29910</v>
@@ -1841,7 +1841,7 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>29690.34</v>
+        <v>29736.59</v>
       </c>
       <c r="B20" s="2" t="n">
         <v>29970</v>
@@ -1870,7 +1870,7 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>29695.34</v>
+        <v>29741.59</v>
       </c>
       <c r="B21" s="2" t="n">
         <v>29975</v>
@@ -1903,7 +1903,7 @@
     </row>
     <row r="22">
       <c r="A22" s="5" t="n">
-        <v>29710.34</v>
+        <v>29756.59</v>
       </c>
       <c r="B22" s="5" t="n">
         <v>29990</v>
@@ -1936,7 +1936,7 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>29713.87</v>
+        <v>29760.12</v>
       </c>
       <c r="B23" s="2" t="n">
         <v>730</v>
@@ -1965,7 +1965,7 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>29796.05</v>
+        <v>29842.3</v>
       </c>
       <c r="B24" s="2" t="n">
         <v>732</v>
@@ -1994,7 +1994,7 @@
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>29919.31</v>
+        <v>29965.56</v>
       </c>
       <c r="B25" s="2" t="n">
         <v>735</v>
@@ -2023,7 +2023,7 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>30001.48</v>
+        <v>30047.73</v>
       </c>
       <c r="B26" s="2" t="n">
         <v>737</v>
@@ -2407,7 +2407,7 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>91.29000000000001</v>
+        <v>91.33</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>150</v>
@@ -2436,7 +2436,7 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>94.34</v>
+        <v>94.38</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>155</v>
@@ -2465,7 +2465,7 @@
     </row>
     <row r="4">
       <c r="A4" s="5" t="n">
-        <v>97.38</v>
+        <v>97.42</v>
       </c>
       <c r="B4" s="5" t="n">
         <v>160</v>
@@ -2498,7 +2498,7 @@
     </row>
     <row r="5">
       <c r="A5" s="5" t="n">
-        <v>100.42</v>
+        <v>100.46</v>
       </c>
       <c r="B5" s="5" t="n">
         <v>165</v>
@@ -2531,7 +2531,7 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>101.03</v>
+        <v>101.07</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>166</v>
@@ -2564,7 +2564,7 @@
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
-        <v>102.86</v>
+        <v>102.9</v>
       </c>
       <c r="B7" s="5" t="n">
         <v>169</v>
@@ -2597,7 +2597,7 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>104.68</v>
+        <v>104.73</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>172</v>
@@ -2630,7 +2630,7 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>105.9</v>
+        <v>105.94</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>174</v>
@@ -2659,7 +2659,7 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>106.51</v>
+        <v>106.55</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>175</v>
@@ -2692,7 +2692,7 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>109.55</v>
+        <v>109.6</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>180</v>
@@ -2783,7 +2783,7 @@
     </row>
     <row r="2">
       <c r="A2" s="5" t="n">
-        <v>3957.68</v>
+        <v>3957</v>
       </c>
       <c r="B2" s="5" t="n">
         <v>82</v>
@@ -2816,7 +2816,7 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>3959.48</v>
+        <v>3958.8</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>365</v>
@@ -2845,7 +2845,7 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>3981.18</v>
+        <v>3980.49</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>367</v>
@@ -2878,7 +2878,7 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>3981.82</v>
+        <v>3981.13</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>82.5</v>
@@ -2911,7 +2911,7 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>3992.03</v>
+        <v>3991.34</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>368</v>
@@ -2940,7 +2940,7 @@
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
-        <v>4005.95</v>
+        <v>4005.26</v>
       </c>
       <c r="B7" s="5" t="n">
         <v>83</v>
@@ -2973,7 +2973,7 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>4030.08</v>
+        <v>4029.38</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>83.5</v>
@@ -3006,7 +3006,7 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>4046.27</v>
+        <v>4045.57</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>373</v>
@@ -3035,7 +3035,7 @@
     </row>
     <row r="10">
       <c r="A10" s="5" t="n">
-        <v>4067.96</v>
+        <v>4067.26</v>
       </c>
       <c r="B10" s="5" t="n">
         <v>375</v>
@@ -3068,7 +3068,7 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>4100.51</v>
+        <v>4099.8</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>378</v>
@@ -3097,7 +3097,7 @@
     </row>
     <row r="12">
       <c r="A12" s="5" t="n">
-        <v>4102.48</v>
+        <v>4101.77</v>
       </c>
       <c r="B12" s="5" t="n">
         <v>85</v>
@@ -3130,7 +3130,7 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>4111.36</v>
+        <v>4110.64</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>379</v>
@@ -3163,7 +3163,7 @@
     </row>
     <row r="14">
       <c r="A14" s="5" t="n">
-        <v>4122.2</v>
+        <v>4121.49</v>
       </c>
       <c r="B14" s="5" t="n">
         <v>380</v>
@@ -3196,7 +3196,7 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>4165.59</v>
+        <v>4164.87</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>384</v>
@@ -3225,7 +3225,7 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>4174.87</v>
+        <v>4174.15</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>86.5</v>
@@ -3258,7 +3258,7 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>4187.29</v>
+        <v>4186.57</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>386</v>
@@ -3287,7 +3287,7 @@
     </row>
     <row r="18">
       <c r="A18" s="5" t="n">
-        <v>4199.01</v>
+        <v>4198.28</v>
       </c>
       <c r="B18" s="5" t="n">
         <v>87</v>
@@ -3320,7 +3320,7 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>4343.8</v>
+        <v>4343.05</v>
       </c>
       <c r="B19" s="2" t="n">
         <v>90</v>
@@ -3510,12 +3510,12 @@
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>-$16.70M</t>
+          <t>-$16.48M</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>+$40.44M</t>
+          <t>+$39.90M</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -3536,7 +3536,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>4102.48</v>
+        <v>4101.77</v>
       </c>
       <c r="C5" s="5" t="n">
         <v>85</v>
@@ -3624,12 +3624,12 @@
       </c>
       <c r="E7" s="9" t="inlineStr">
         <is>
-          <t>+$7.82M</t>
+          <t>+$7.59M</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>+$23.22M</t>
+          <t>+$22.53M</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
@@ -3662,12 +3662,12 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>-$3.95M</t>
+          <t>-$3.85M</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>+$21.70M</t>
+          <t>+$21.18M</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
@@ -3722,7 +3722,7 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>3957.68</v>
+        <v>3957</v>
       </c>
       <c r="C10" s="5" t="n">
         <v>82</v>
@@ -3798,7 +3798,7 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>29508.44</v>
+        <v>29554.69</v>
       </c>
       <c r="C12" s="5" t="n">
         <v>725</v>
@@ -3874,24 +3874,24 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>7705.28</v>
+        <v>7654.52</v>
       </c>
       <c r="C14" s="5" t="n">
-        <v>768</v>
+        <v>7650</v>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="E14" s="9" t="inlineStr">
-        <is>
-          <t>+$3.64M</t>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E14" s="7" t="inlineStr">
+        <is>
+          <t>-$9.17M</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>+$12.17M</t>
+          <t>+$12.20M</t>
         </is>
       </c>
       <c r="G14" s="6" t="inlineStr">
@@ -3901,7 +3901,7 @@
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>peak</t>
+          <t>valley</t>
         </is>
       </c>
     </row>
@@ -3912,24 +3912,24 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>7654.52</v>
+        <v>7705.28</v>
       </c>
       <c r="C15" s="5" t="n">
-        <v>7650</v>
+        <v>768</v>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E15" s="7" t="inlineStr">
-        <is>
-          <t>-$8.65M</t>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>+$3.64M</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>+$11.50M</t>
+          <t>+$12.17M</t>
         </is>
       </c>
       <c r="G15" s="6" t="inlineStr">
@@ -3939,7 +3939,7 @@
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>valley</t>
+          <t>peak</t>
         </is>
       </c>
     </row>
@@ -4038,12 +4038,12 @@
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>+$8.02M</t>
+          <t>+$7.83M</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>+$11.11M</t>
+          <t>+$10.84M</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -4058,78 +4058,78 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>4005.26</v>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>83</v>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>+$9.47M</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>+$10.16M</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B19" s="2" t="n">
+      <c r="B20" s="2" t="n">
         <v>7724.52</v>
       </c>
-      <c r="C19" s="2" t="n">
+      <c r="C20" s="2" t="n">
         <v>7720</v>
       </c>
-      <c r="D19" s="3" t="inlineStr">
+      <c r="D20" s="3" t="inlineStr">
         <is>
           <t>SPX</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>-$4.14M</t>
-        </is>
-      </c>
-      <c r="F19" s="3" t="inlineStr">
-        <is>
-          <t>+$10.24M</t>
-        </is>
-      </c>
-      <c r="G19" s="3" t="inlineStr">
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>-$4.04M</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>+$9.99M</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
         <is>
           <t>Net</t>
         </is>
       </c>
-      <c r="H19" s="3" t="inlineStr">
+      <c r="H20" s="3" t="inlineStr">
         <is>
           <t>valley</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="n">
-        <v>4005.95</v>
-      </c>
-      <c r="C20" s="5" t="n">
-        <v>83</v>
-      </c>
-      <c r="D20" s="6" t="inlineStr">
-        <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E20" s="9" t="inlineStr">
-        <is>
-          <t>+$9.47M</t>
-        </is>
-      </c>
-      <c r="F20" s="6" t="inlineStr">
-        <is>
-          <t>+$10.16M</t>
-        </is>
-      </c>
-      <c r="G20" s="6" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H20" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
         </is>
       </c>
     </row>
@@ -4140,7 +4140,7 @@
         </is>
       </c>
       <c r="B21" s="5" t="n">
-        <v>4199.01</v>
+        <v>4198.28</v>
       </c>
       <c r="C21" s="5" t="n">
         <v>87</v>
@@ -4190,12 +4190,12 @@
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>-$1.62M</t>
+          <t>-$1.66M</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>+$8.88M</t>
+          <t>+$9.07M</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
@@ -4254,7 +4254,7 @@
         </is>
       </c>
       <c r="B24" s="5" t="n">
-        <v>29220.83</v>
+        <v>29267.08</v>
       </c>
       <c r="C24" s="5" t="n">
         <v>718</v>
@@ -4304,12 +4304,12 @@
       </c>
       <c r="E25" s="8" t="inlineStr">
         <is>
-          <t>+$561.75K</t>
+          <t>+$547.34K</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>+$7.62M</t>
+          <t>+$7.42M</t>
         </is>
       </c>
       <c r="G25" s="3" t="inlineStr">
@@ -4330,7 +4330,7 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>29303</v>
+        <v>29349.25</v>
       </c>
       <c r="C26" s="5" t="n">
         <v>720</v>
@@ -4380,12 +4380,12 @@
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>-$6.07M</t>
+          <t>-$6.76M</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr">
         <is>
-          <t>+$6.54M</t>
+          <t>+$7.25M</t>
         </is>
       </c>
       <c r="G27" s="6" t="inlineStr">
@@ -4406,7 +4406,7 @@
         </is>
       </c>
       <c r="B28" s="2" t="n">
-        <v>29590.61</v>
+        <v>29636.86</v>
       </c>
       <c r="C28" s="2" t="n">
         <v>727</v>
@@ -4440,7 +4440,7 @@
         </is>
       </c>
       <c r="B29" s="2" t="n">
-        <v>29097.57</v>
+        <v>29143.82</v>
       </c>
       <c r="C29" s="2" t="n">
         <v>715</v>
@@ -4486,12 +4486,12 @@
       </c>
       <c r="E30" s="8" t="inlineStr">
         <is>
-          <t>+$1.73M</t>
+          <t>+$1.70M</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>+$5.62M</t>
+          <t>+$5.52M</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
@@ -4512,7 +4512,7 @@
         </is>
       </c>
       <c r="B31" s="2" t="n">
-        <v>29713.87</v>
+        <v>29760.12</v>
       </c>
       <c r="C31" s="2" t="n">
         <v>730</v>
@@ -4546,7 +4546,7 @@
         </is>
       </c>
       <c r="B32" s="2" t="n">
-        <v>29385.18</v>
+        <v>29431.43</v>
       </c>
       <c r="C32" s="2" t="n">
         <v>722</v>
@@ -4614,7 +4614,7 @@
         </is>
       </c>
       <c r="B34" s="2" t="n">
-        <v>29056.48</v>
+        <v>29102.73</v>
       </c>
       <c r="C34" s="2" t="n">
         <v>714</v>
@@ -4652,7 +4652,7 @@
         </is>
       </c>
       <c r="B35" s="5" t="n">
-        <v>102.86</v>
+        <v>102.9</v>
       </c>
       <c r="C35" s="5" t="n">
         <v>169</v>
@@ -4778,12 +4778,12 @@
       </c>
       <c r="E38" s="8" t="inlineStr">
         <is>
-          <t>+$1.05M</t>
+          <t>+$1.02M</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>+$4.25M</t>
+          <t>+$4.09M</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
@@ -4804,7 +4804,7 @@
         </is>
       </c>
       <c r="B39" s="2" t="n">
-        <v>4343.8</v>
+        <v>4343.05</v>
       </c>
       <c r="C39" s="2" t="n">
         <v>90</v>
@@ -4838,7 +4838,7 @@
         </is>
       </c>
       <c r="B40" s="2" t="n">
-        <v>28892.13</v>
+        <v>28938.38</v>
       </c>
       <c r="C40" s="2" t="n">
         <v>710</v>
@@ -4872,7 +4872,7 @@
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>100.42</v>
+        <v>100.46</v>
       </c>
       <c r="C41" s="5" t="n">
         <v>165</v>
@@ -4910,7 +4910,7 @@
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>29261.92</v>
+        <v>29308.17</v>
       </c>
       <c r="C42" s="2" t="n">
         <v>719</v>
@@ -4948,7 +4948,7 @@
         </is>
       </c>
       <c r="B43" s="2" t="n">
-        <v>29796.05</v>
+        <v>29842.3</v>
       </c>
       <c r="C43" s="2" t="n">
         <v>732</v>
@@ -5012,36 +5012,40 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B45" s="2" t="n">
-        <v>29919.31</v>
+        <v>7649.52</v>
       </c>
       <c r="C45" s="2" t="n">
-        <v>735</v>
+        <v>7645</v>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E45" s="8" t="inlineStr">
-        <is>
-          <t>+$2.21M</t>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>-$1.76M</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>+$2.40M</t>
+          <t>+$2.45M</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
         <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H45" s="3" t="inlineStr"/>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>peak</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
@@ -5050,62 +5054,58 @@
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>29138.65</v>
+        <v>29965.56</v>
       </c>
       <c r="C46" s="2" t="n">
-        <v>716</v>
+        <v>735</v>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
           <t>QQQ</t>
         </is>
       </c>
-      <c r="E46" s="4" t="inlineStr">
-        <is>
-          <t>-$845.19K</t>
+      <c r="E46" s="8" t="inlineStr">
+        <is>
+          <t>+$2.21M</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>+$2.39M</t>
+          <t>+$2.40M</t>
         </is>
       </c>
       <c r="G46" s="3" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H46" s="3" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H46" s="3" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B47" s="2" t="n">
-        <v>7649.52</v>
+        <v>29184.9</v>
       </c>
       <c r="C47" s="2" t="n">
-        <v>7645</v>
+        <v>716</v>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>SPX</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>-$1.71M</t>
+          <t>-$845.19K</t>
         </is>
       </c>
       <c r="F47" s="3" t="inlineStr">
         <is>
-          <t>+$2.37M</t>
+          <t>+$2.39M</t>
         </is>
       </c>
       <c r="G47" s="3" t="inlineStr">
@@ -5126,7 +5126,7 @@
         </is>
       </c>
       <c r="B48" s="2" t="n">
-        <v>30001.48</v>
+        <v>30047.73</v>
       </c>
       <c r="C48" s="2" t="n">
         <v>737</v>
@@ -5160,7 +5160,7 @@
         </is>
       </c>
       <c r="B49" s="2" t="n">
-        <v>105.9</v>
+        <v>105.94</v>
       </c>
       <c r="C49" s="2" t="n">
         <v>174</v>
@@ -5194,7 +5194,7 @@
         </is>
       </c>
       <c r="B50" s="2" t="n">
-        <v>28809.96</v>
+        <v>28856.21</v>
       </c>
       <c r="C50" s="2" t="n">
         <v>708</v>
@@ -5228,7 +5228,7 @@
         </is>
       </c>
       <c r="B51" s="5" t="n">
-        <v>97.38</v>
+        <v>97.42</v>
       </c>
       <c r="C51" s="5" t="n">
         <v>160</v>
@@ -5266,7 +5266,7 @@
         </is>
       </c>
       <c r="B52" s="2" t="n">
-        <v>28686.7</v>
+        <v>28732.95</v>
       </c>
       <c r="C52" s="2" t="n">
         <v>705</v>
@@ -5300,7 +5300,7 @@
         </is>
       </c>
       <c r="B53" s="5" t="n">
-        <v>4122.2</v>
+        <v>4121.49</v>
       </c>
       <c r="C53" s="5" t="n">
         <v>380</v>
@@ -5338,7 +5338,7 @@
         </is>
       </c>
       <c r="B54" s="2" t="n">
-        <v>101.03</v>
+        <v>101.07</v>
       </c>
       <c r="C54" s="2" t="n">
         <v>166</v>
@@ -5376,7 +5376,7 @@
         </is>
       </c>
       <c r="B55" s="2" t="n">
-        <v>106.51</v>
+        <v>106.55</v>
       </c>
       <c r="C55" s="2" t="n">
         <v>175</v>
@@ -5490,7 +5490,7 @@
         </is>
       </c>
       <c r="B58" s="5" t="n">
-        <v>4067.96</v>
+        <v>4067.26</v>
       </c>
       <c r="C58" s="5" t="n">
         <v>375</v>
@@ -5528,7 +5528,7 @@
         </is>
       </c>
       <c r="B59" s="2" t="n">
-        <v>4174.87</v>
+        <v>4174.15</v>
       </c>
       <c r="C59" s="2" t="n">
         <v>86.5</v>
@@ -5566,7 +5566,7 @@
         </is>
       </c>
       <c r="B60" s="2" t="n">
-        <v>4046.27</v>
+        <v>4045.57</v>
       </c>
       <c r="C60" s="2" t="n">
         <v>373</v>
@@ -5600,7 +5600,7 @@
         </is>
       </c>
       <c r="B61" s="2" t="n">
-        <v>94.34</v>
+        <v>94.38</v>
       </c>
       <c r="C61" s="2" t="n">
         <v>155</v>
@@ -5634,7 +5634,7 @@
         </is>
       </c>
       <c r="B62" s="2" t="n">
-        <v>3992.03</v>
+        <v>3991.34</v>
       </c>
       <c r="C62" s="2" t="n">
         <v>368</v>
@@ -5668,7 +5668,7 @@
         </is>
       </c>
       <c r="B63" s="5" t="n">
-        <v>29710.34</v>
+        <v>29756.59</v>
       </c>
       <c r="C63" s="5" t="n">
         <v>29990</v>
@@ -5706,7 +5706,7 @@
         </is>
       </c>
       <c r="B64" s="2" t="n">
-        <v>4100.51</v>
+        <v>4099.8</v>
       </c>
       <c r="C64" s="2" t="n">
         <v>378</v>
@@ -5740,7 +5740,7 @@
         </is>
       </c>
       <c r="B65" s="2" t="n">
-        <v>104.68</v>
+        <v>104.73</v>
       </c>
       <c r="C65" s="2" t="n">
         <v>172</v>
@@ -5778,7 +5778,7 @@
         </is>
       </c>
       <c r="B66" s="2" t="n">
-        <v>3959.48</v>
+        <v>3958.8</v>
       </c>
       <c r="C66" s="2" t="n">
         <v>365</v>
@@ -5812,7 +5812,7 @@
         </is>
       </c>
       <c r="B67" s="2" t="n">
-        <v>3981.18</v>
+        <v>3980.49</v>
       </c>
       <c r="C67" s="2" t="n">
         <v>367</v>
@@ -5850,7 +5850,7 @@
         </is>
       </c>
       <c r="B68" s="2" t="n">
-        <v>109.55</v>
+        <v>109.6</v>
       </c>
       <c r="C68" s="2" t="n">
         <v>180</v>
@@ -5884,7 +5884,7 @@
         </is>
       </c>
       <c r="B69" s="2" t="n">
-        <v>91.29000000000001</v>
+        <v>91.33</v>
       </c>
       <c r="C69" s="2" t="n">
         <v>150</v>
@@ -5918,7 +5918,7 @@
         </is>
       </c>
       <c r="B70" s="2" t="n">
-        <v>4187.29</v>
+        <v>4186.57</v>
       </c>
       <c r="C70" s="2" t="n">
         <v>386</v>
@@ -5952,7 +5952,7 @@
         </is>
       </c>
       <c r="B71" s="2" t="n">
-        <v>4111.36</v>
+        <v>4110.64</v>
       </c>
       <c r="C71" s="2" t="n">
         <v>379</v>
@@ -5990,7 +5990,7 @@
         </is>
       </c>
       <c r="B72" s="2" t="n">
-        <v>3981.82</v>
+        <v>3981.13</v>
       </c>
       <c r="C72" s="2" t="n">
         <v>82.5</v>
@@ -6028,7 +6028,7 @@
         </is>
       </c>
       <c r="B73" s="5" t="n">
-        <v>29380.34</v>
+        <v>29426.59</v>
       </c>
       <c r="C73" s="5" t="n">
         <v>29660</v>
@@ -6066,7 +6066,7 @@
         </is>
       </c>
       <c r="B74" s="2" t="n">
-        <v>4165.59</v>
+        <v>4164.87</v>
       </c>
       <c r="C74" s="2" t="n">
         <v>384</v>
@@ -6100,7 +6100,7 @@
         </is>
       </c>
       <c r="B75" s="2" t="n">
-        <v>4030.08</v>
+        <v>4029.38</v>
       </c>
       <c r="C75" s="2" t="n">
         <v>83.5</v>
@@ -6138,7 +6138,7 @@
         </is>
       </c>
       <c r="B76" s="5" t="n">
-        <v>29630.34</v>
+        <v>29676.59</v>
       </c>
       <c r="C76" s="5" t="n">
         <v>29910</v>
@@ -6176,7 +6176,7 @@
         </is>
       </c>
       <c r="B77" s="5" t="n">
-        <v>29440.34</v>
+        <v>29486.59</v>
       </c>
       <c r="C77" s="5" t="n">
         <v>29720</v>
@@ -6214,7 +6214,7 @@
         </is>
       </c>
       <c r="B78" s="2" t="n">
-        <v>29690.34</v>
+        <v>29736.59</v>
       </c>
       <c r="C78" s="2" t="n">
         <v>29970</v>
@@ -6248,7 +6248,7 @@
         </is>
       </c>
       <c r="B79" s="2" t="n">
-        <v>29530.34</v>
+        <v>29576.59</v>
       </c>
       <c r="C79" s="2" t="n">
         <v>29810</v>
@@ -6282,7 +6282,7 @@
         </is>
       </c>
       <c r="B80" s="2" t="n">
-        <v>29410.34</v>
+        <v>29456.59</v>
       </c>
       <c r="C80" s="2" t="n">
         <v>29690</v>
@@ -6320,7 +6320,7 @@
         </is>
       </c>
       <c r="B81" s="2" t="n">
-        <v>29510.34</v>
+        <v>29556.59</v>
       </c>
       <c r="C81" s="2" t="n">
         <v>29790</v>
@@ -6358,7 +6358,7 @@
         </is>
       </c>
       <c r="B82" s="2" t="n">
-        <v>29695.34</v>
+        <v>29741.59</v>
       </c>
       <c r="C82" s="2" t="n">
         <v>29975</v>

</xml_diff>